<commit_message>
Combined scan results 2026-10-06
</commit_message>
<xml_diff>
--- a/results/2026-10-06.xlsx
+++ b/results/2026-10-06.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,10 +445,14 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ECHO</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>AAOI</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -459,7 +463,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>ALAB</t>
         </is>
       </c>
     </row>
@@ -467,7 +471,7 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AIP</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -491,13 +495,13 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ACMR</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>ANGO</t>
         </is>
       </c>
     </row>
@@ -505,18 +509,18 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ATAT</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>AEHR</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
@@ -524,18 +528,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAPR</t>
+          <t>COST</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AEHR</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BAND</t>
+          <t>BGC</t>
         </is>
       </c>
     </row>
@@ -543,18 +547,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CHRW</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ALNT</t>
+          <t>ARW</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CORT</t>
+          <t>CHEF</t>
         </is>
       </c>
     </row>
@@ -562,209 +566,305 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>CRDO</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>HON</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ARW</t>
+          <t>AVPT</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>CRWD</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>IBOC</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>AVT</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>DGII</t>
+          <t>CVCO</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>IDXX</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>AXTI</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>DXPE</t>
+          <t>DDOG</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>LIN</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AVT</t>
+          <t>CAKE</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>FFIV</t>
+          <t>EXEL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>MKSI</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AXTI</t>
+          <t>CAMT</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>FORM</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MYRG</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>CDNA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>ILMN</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>NTES</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>CGNX</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>IOVA</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>NVTS</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CEVA</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>IRDM</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PECO</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CHEF</t>
+          <t>COHU</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>KOD</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>POET</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>CORT</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LGND</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>POWL</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>COHU</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LILAK</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PWP</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>CRAI</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>MAR</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>RYAAY</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CVCO</t>
+          <t>CVLT</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>MEDP</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>STRL</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>CYRX</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SUPN</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>DIOD</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>MRX</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
@@ -775,7 +875,11 @@
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>PAYO</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
@@ -786,62 +890,626 @@
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>QMCO</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>FFIV</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>SBLK</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>FOSL</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SHOO</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>FOSL</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SIMO</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>FRHC</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SMTC</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
+          <t>FROG</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>VICR</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>FTNT</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>GH</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>XMTR</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>GRAL</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>GSAT</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
           <t>HIMX</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>IBRX</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ICHR</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>IDCC</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>IESC</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>KLIC</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>LAUR</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>LECO</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>LFUS</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>LIND</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>LITE</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>LSCC</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>MPWR</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>MTSI</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>MXL</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>NDSN</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>NNBR</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>NTAP</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>NTNX</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>OKTA</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr"/>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr"/>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>PAYS</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr"/>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>PCVX</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>PENG</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr"/>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>PLXS</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>PRCH</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>QLYS</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr"/>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>RVMD</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>SANM</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr"/>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>SCSC</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr"/>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr"/>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>SITM</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr"/>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>SLAB</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr"/>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>SYNA</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr"/>
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr"/>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>TRMD</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr"/>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>VCTR</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -854,7 +1522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -882,374 +1550,198 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AEHR</t>
+          <t>PTC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ABCL</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AMKR</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>GMAB</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>SDEV</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ABSI</t>
+          <t>RXRX</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FLY</t>
+          <t>MDLN</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>CRDO</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AVT</t>
+          <t>ILMN</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MDLN</t>
+          <t>ASST</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>GTLB</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AXTI</t>
+          <t>KOD</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>IBRX</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>OUST</t>
+          <t>MRNA</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>NVAX</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>IOVA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>RKLB</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>MSTR</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>COHU</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>MCHP</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>META</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>QMCO</t>
+          <t>NTNX</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>PENG</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>MXL</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SAIL</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>TRMD</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>SDGR</t>
+          <t>PACB</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>XRPN</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BMNR</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>FPS</t>
+          <t>SDGR</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>SMCI</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>FTNT</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>SUNB</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>FRSH</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>SMTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>LAUR</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>FORM</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>KLAC</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>MAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>LIND</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>IBRX</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>KOD</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>NBIS</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>LITE</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>LSCC</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>MCHP</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>NTNX</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>META</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>MXL</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>MGNI</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>NVAX</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>MRVL</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>NTAP</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>OLLI</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>PANW</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>SHOO</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>NVDA</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>PLTR</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>RMBS</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>TENB</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>PACB</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>OKTA</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>SHLS</t>
+          <t>SKHY</t>
         </is>
       </c>
     </row>

</xml_diff>